<commit_message>
Author Ledger Europe: partial results; allow author-domain contact emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/author-ledger/europe/Author_Ledger_Europe_Leads.xlsx
+++ b/author-ledger/europe/Author_Ledger_Europe_Leads.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COUNTRY PROGRESS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'READY'!$A$1:$S$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NEEDS REVIEW'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'READY'!$A$1:$S$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NEEDS REVIEW'!$A$1:$S$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DUPLICATES'!$A$1:$S$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -558,8 +558,384 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tuomas Niskakangas</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The Sealed Case (Department K series, book 1)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Crime</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>satu@ahlbackagency.com</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/about-us/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/2026/03/19/second-pre-publication-deal-fortuomas-niskakangas-new-series/</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026 pre-publication deals: German (Bastei Lübbe, first two books) and Greek (Memento, full trilogy)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>New Department K crime trilogy sold pre-publication to Bastei Lübbe and Memento in 2026</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>High - new crime trilogy with pre-publication foreign deals</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Finnish</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Verify Finnish publisher and exact 2026 pub date; Satu Sallantaus closed Greek deal, Martti Berner the German one</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ingar Johnsrud</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>De svarte enkene (The Black Widows)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Thriller</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>evy.tillman@osloliteraryagency.no</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://osloliteraryagency.no/this-is-us-2/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://osloliteraryagency.no/author/ingar-johnsrud/</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Aschehoug</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://osloliteraryagency.no/wp-content/uploads/sites/81/2025/09/Katalog-Fiction-Non-Fiction-Autumn-2025-WEB.pdf</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>New thriller August 2025 on Oslo Literary Agency Autumn 2025 rights list</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Former crime journalist whose debut was The Vienna Brotherhood (2015); The Black Widows is a 395-page thriller</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>High - established translated thriller series author, mid-list internationally</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Norwegian</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Confirm assigned agent at Oslo Literary Agency (Evy Tillman vs Henrik Francke henrik@osloliteraryagency.no)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sven Petter Næss</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>I dødsonen (Dead Zone)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Crime</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>evy.tillman@osloliteraryagency.no</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://osloliteraryagency.no/this-is-us-2/</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://osloliteraryagency.no/author/sven-p-n/</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Aschehoug</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://osloliteraryagency.no/wp-content/uploads/sites/81/2025/09/Katalog-Fiction-Non-Fiction-Autumn-2025-WEB.pdf</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Listed on Oslo Literary Agency Autumn 2025 rights list; author page lists a 2026 title, Black Holes</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Dead Zone: a Norwegian man in London is arrested for murder after a woman is found hanged near his home</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>High - Nordic crime with London setting, follow-up 2026 title</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Norwegian</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Agent email is Oslo Literary Agency contact (Evy Tillman; rights lists also show evy@ / henrik@); confirm which agent handles Næss</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Katarzyna Puzyńska</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dzielnica cieni (Zalesie series)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Crime fiction</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>kontakt@katarzynapuzynska.pl</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.katarzynapuzynska.pl/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.katarzynapuzynska.pl/</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://lubimyczytac.pl/autor/95374/katarzyna-puzynska</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>New Zalesie crime series; Dziennik.pl reported her return with a new book</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Launched a new crime series, Zalesie, after her long-running bestselling series (per Dziennik.pl / lubimyczytac)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>High - bestselling Polish crime author with an active new series</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Email is kontakt@ on the author's own domain (not a third-party generic); confirm the Dzielnica cieni 2025 date and the publisher (likely Prószyński); she may be too big for the mid-list target</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S1"/>
+  <autoFilter ref="A1:S5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -570,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -691,8 +1067,842 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Michaela Klevisová</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Letní slunovrat</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Crime fiction</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>http://www.michaelaklevisova.cz/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Motto</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.databazeknih.cz/autori/michaela-klevisova-10709</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Published Letní slunovrat (Motto, 2025)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Letní slunovrat is a crime novel set in a South Bohemian village</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>High - established Czech crime novelist</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Czech</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Find a contact or press email on michaelaklevisova.cz or motto.cz | Review: no valid email; email type missing; No email found; check the author's site or Motto's press contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Veronika Martinková</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pohřbena zaživa</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Crime fiction</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://veronikamartinkova.cz/</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>VM knihy (self-published)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.centrum-detektivky.cz/autori/veronika-martinkova</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Sebevražda (2025) and Pohřbena zaživa (2026), self-published through VM knihy</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Brno-based crime writer who publishes her own books through her own house, VM knihy</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>High - prolific indie crime author with yearly releases</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Czech</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Check the contact page for a non-billing author or press email | Review: no valid email; email type missing; Only a billing address (fakturace@vmknihy.cz) appeared in search results; it is not acceptable. Need a contact email from the veronikamartinkova.cz/kontakt page</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jesper Bugge Kold</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Where the Fire Burns</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.nordinagency.se/the-mofibo-awards-nominations-are-out-in-denmark/</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2025: book out in Denmark; nominated for Author of the Year Award</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Where the Fire Burns out in Denmark 2025; Author of the Year nomination</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Medium - nominated Danish author with Nordin Ringhof representation</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Danish</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Find Lars Ringhof / Anna Richter email on nordinagency.se/contact | Review: no valid email; email type missing; No agent email tied to author found (Nordin Ringhof Copenhagen staff emails not visible in snippets)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ann-Luise Bertell</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A Heart With Two Minds</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fiction</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>satu@ahlbackagency.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/about-us/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/2026/09/14/a-heart-with-two-minds-albanian-language-rights-sold/</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Sept 2026: Albanian rights sold to Justina Prima</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>A Heart With Two Minds sold to Albania in Sept 2026</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Medium - Finland-Swedish fiction with ongoing rights sales</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Swedish</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Finland-Swedish author; verify pub year and language | Review: no 2025–2027 publication date; Original publication date unconfirmed; genre/premise not sourced</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Annukka Salama</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The Melting Point</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>YA romance (queer hockey romance)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>noora@ahlbackagency.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/about-us/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/2026/03/05/three-deals-for-annukka-salamas-the-melting-point-in-one-day/</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026: German rights at auction (Bastei Lübbe ONE), Dutch, French, Swedish, Spanish, Estonian, Ukrainian deals; first deal for new title TAKEN WILD (Aug 2026)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Queer YA hockey romance The Melting Point sold at auction in Germany in May 2026</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>High - hot YA romance with many 2026 rights sales</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Finnish</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Confirm Finnish pub year/publisher; Noora Al-Ani closed French/Swedish/Spanish deals | Review: no 2025–2027 publication date; Finnish publication date of The Melting Point not shown in snippets</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tommi Kinnunen</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Defiance</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Literary fiction</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>satu@ahlbackagency.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/about-us/</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://www.ahlbackagency.com/2026/09/28/ukrainian-rights-for-defiance-by-tommi-kinnunen-sold/</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Sept 2026: Ukrainian rights to Defiance sold to Booksetter, 10th foreign deal</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Defiance reached its 10th foreign-rights deal in Sept 2026</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Medium - literary fiction with strong international reach</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Finnish</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Check Defiance Finnish pub year; Satu Sallantaus closed the deal | Review: no 2025–2027 publication date; Original publication date of Defiance unconfirmed (may predate 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Izabela Janiszewska</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Zamknięte w lodzie</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Crime fiction</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://kultura.dziennik.pl/ksiazki/artykuly/11244110,autorka-bestsellerowych-kryminalow-powraca-z-nowa-seria-zapowiada-sie-hit.html</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Starting a new crime series with Zamknięte w lodzie</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Zamknięte w lodzie opens her new crime series (Dziennik.pl)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>High - bestselling crime author launching a new series</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Confirm the 2025/2026 date and find an agent or publisher press email | Review: no valid email; email type missing; no 2025–2027 publication date; No email, website or confirmed date/publisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Katarzyna Romanowska</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>His Obsession (Polish title unconfirmed)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Romance (likely)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://czytamdo.pl/2025/10/07/kto-tu-ma-obsesje-katarzyna-romanowska-walczy-z-booktokiem/</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>In Sep 2025 drew attention by openly responding to negative BookTok reviews</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Novel released June 2025; the BookTok controversy over her responses to reviews grew in September 2025</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Low - reputational controversy; genre unconfirmed</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Check the controversy before any outreach; probably deprioritise | Review: no valid email; email type missing; No email, publisher or genre confirmation; controversy risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Paulina Świst</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>UMBRA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Crime fiction / romantic suspense</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>kontakt@paulinaswist.pl</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>http://paulinaswist.pl/kontakt/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://paulinaswist.pl/</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://paulinaswist.pl/ksiazki/</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Official site lists UMBRA as her newest crime novel</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Her About page says she rarely gives interviews, even by phone</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>High - popular Polish commercial crime/romance author</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Confirm UMBRA's release date and publisher; email is from the author's official contact page | Review: no 2025–2027 publication date; UMBRA's publication year (2025/2026) is not confirmed in search text; publisher unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>William Älgebrink</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Huset vid Pärlälvens slut (The House by Pearl River)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Psychological suspense / crime</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>johanna.lindborg@bonnierrights.se</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://bonnierrights.se/contact/william-algebrink/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Romanus &amp; Selling</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://bonnierrights.se/contact/william-algebrink/</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Won CrimeTime Award for Best Crime Debut of the Year, October 2025</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>CrimeTime jury called the debut a dizzying descent into darkness set against the Norrbotten forest</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>High - award-winning crime debut</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Swedish</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>NEEDS REVIEW</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Johanna Lindborg named as foreign rights contact on author page; email from Bonnier Rights agent listing | Review: no 2025–2027 publication date; Book published Oct 2024; need confirmed 2025/2026/2027 follow-up title</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S1"/>
+  <autoFilter ref="A1:S11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -836,7 +2046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -880,27 +2090,177 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Czechia</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="3" t="n">
+      <c r="B8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>